<commit_message>
Referral template: drop address + payment method fields
Remove Payment Method column from the log (and its dropdown), the payee
Address field from the voucher, and the Payment Method lines from voucher
and receipt. Also strip em dashes from sample text.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WYLXC9uaFEEBGfEAmw5PKy
</commit_message>
<xml_diff>
--- a/Referral_Fee_Log_Voucher_Receipt.xlsx
+++ b/Referral_Fee_Log_Voucher_Receipt.xlsx
@@ -90,7 +90,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -161,11 +161,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -200,6 +215,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -602,6 +619,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -609,6 +627,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
@@ -647,20 +666,15 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Payment Method</t>
+          <t>Payment Ref</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Payment Ref</t>
+          <t>Receipt No.</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>Receipt No.</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Running Total (RM)</t>
         </is>
@@ -692,7 +706,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Umesh Phadke — AB-39-02 MK 10</t>
+          <t>Umesh Phadke, AB-39-02 MK 10</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -700,20 +714,15 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>TXN12345</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>TXN12345</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
           <t>OR/2026/001</t>
         </is>
       </c>
-      <c r="K8" s="7">
+      <c r="J8" s="7">
         <f>IF(G8="","",SUM($G$8:G8))</f>
         <v/>
       </c>
@@ -744,7 +753,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Tenant referral — Sunway Palmville</t>
+          <t>Tenant referral, Sunway Palmville</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -752,20 +761,15 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Cheque</t>
+          <t>CHQ000123</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>CHQ000123</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
           <t>OR/2026/002</t>
         </is>
       </c>
-      <c r="K9" s="7">
+      <c r="J9" s="7">
         <f>IF(G9="","",SUM($G$8:G9))</f>
         <v/>
       </c>
@@ -786,8 +790,7 @@
       <c r="G10" s="10" t="n"/>
       <c r="H10" s="8" t="n"/>
       <c r="I10" s="8" t="n"/>
-      <c r="J10" s="8" t="n"/>
-      <c r="K10" s="10">
+      <c r="J10" s="10">
         <f>IF(G10="","",SUM($G$8:G10))</f>
         <v/>
       </c>
@@ -808,8 +811,7 @@
       <c r="G11" s="10" t="n"/>
       <c r="H11" s="8" t="n"/>
       <c r="I11" s="8" t="n"/>
-      <c r="J11" s="8" t="n"/>
-      <c r="K11" s="10">
+      <c r="J11" s="10">
         <f>IF(G11="","",SUM($G$8:G11))</f>
         <v/>
       </c>
@@ -830,8 +832,7 @@
       <c r="G12" s="10" t="n"/>
       <c r="H12" s="8" t="n"/>
       <c r="I12" s="8" t="n"/>
-      <c r="J12" s="8" t="n"/>
-      <c r="K12" s="10">
+      <c r="J12" s="10">
         <f>IF(G12="","",SUM($G$8:G12))</f>
         <v/>
       </c>
@@ -852,8 +853,7 @@
       <c r="G13" s="10" t="n"/>
       <c r="H13" s="8" t="n"/>
       <c r="I13" s="8" t="n"/>
-      <c r="J13" s="8" t="n"/>
-      <c r="K13" s="10">
+      <c r="J13" s="10">
         <f>IF(G13="","",SUM($G$8:G13))</f>
         <v/>
       </c>
@@ -874,8 +874,7 @@
       <c r="G14" s="10" t="n"/>
       <c r="H14" s="8" t="n"/>
       <c r="I14" s="8" t="n"/>
-      <c r="J14" s="8" t="n"/>
-      <c r="K14" s="10">
+      <c r="J14" s="10">
         <f>IF(G14="","",SUM($G$8:G14))</f>
         <v/>
       </c>
@@ -896,8 +895,7 @@
       <c r="G15" s="10" t="n"/>
       <c r="H15" s="8" t="n"/>
       <c r="I15" s="8" t="n"/>
-      <c r="J15" s="8" t="n"/>
-      <c r="K15" s="10">
+      <c r="J15" s="10">
         <f>IF(G15="","",SUM($G$8:G15))</f>
         <v/>
       </c>
@@ -918,8 +916,7 @@
       <c r="G16" s="10" t="n"/>
       <c r="H16" s="8" t="n"/>
       <c r="I16" s="8" t="n"/>
-      <c r="J16" s="8" t="n"/>
-      <c r="K16" s="10">
+      <c r="J16" s="10">
         <f>IF(G16="","",SUM($G$8:G16))</f>
         <v/>
       </c>
@@ -940,8 +937,7 @@
       <c r="G17" s="10" t="n"/>
       <c r="H17" s="8" t="n"/>
       <c r="I17" s="8" t="n"/>
-      <c r="J17" s="8" t="n"/>
-      <c r="K17" s="10">
+      <c r="J17" s="10">
         <f>IF(G17="","",SUM($G$8:G17))</f>
         <v/>
       </c>
@@ -962,8 +958,7 @@
       <c r="G18" s="10" t="n"/>
       <c r="H18" s="8" t="n"/>
       <c r="I18" s="8" t="n"/>
-      <c r="J18" s="8" t="n"/>
-      <c r="K18" s="10">
+      <c r="J18" s="10">
         <f>IF(G18="","",SUM($G$8:G18))</f>
         <v/>
       </c>
@@ -984,8 +979,7 @@
       <c r="G19" s="10" t="n"/>
       <c r="H19" s="8" t="n"/>
       <c r="I19" s="8" t="n"/>
-      <c r="J19" s="8" t="n"/>
-      <c r="K19" s="10">
+      <c r="J19" s="10">
         <f>IF(G19="","",SUM($G$8:G19))</f>
         <v/>
       </c>
@@ -1006,8 +1000,7 @@
       <c r="G20" s="10" t="n"/>
       <c r="H20" s="8" t="n"/>
       <c r="I20" s="8" t="n"/>
-      <c r="J20" s="8" t="n"/>
-      <c r="K20" s="10">
+      <c r="J20" s="10">
         <f>IF(G20="","",SUM($G$8:G20))</f>
         <v/>
       </c>
@@ -1028,8 +1021,7 @@
       <c r="G21" s="10" t="n"/>
       <c r="H21" s="8" t="n"/>
       <c r="I21" s="8" t="n"/>
-      <c r="J21" s="8" t="n"/>
-      <c r="K21" s="10">
+      <c r="J21" s="10">
         <f>IF(G21="","",SUM($G$8:G21))</f>
         <v/>
       </c>
@@ -1050,8 +1042,7 @@
       <c r="G22" s="10" t="n"/>
       <c r="H22" s="8" t="n"/>
       <c r="I22" s="8" t="n"/>
-      <c r="J22" s="8" t="n"/>
-      <c r="K22" s="10">
+      <c r="J22" s="10">
         <f>IF(G22="","",SUM($G$8:G22))</f>
         <v/>
       </c>
@@ -1072,8 +1063,7 @@
       <c r="G23" s="10" t="n"/>
       <c r="H23" s="8" t="n"/>
       <c r="I23" s="8" t="n"/>
-      <c r="J23" s="8" t="n"/>
-      <c r="K23" s="10">
+      <c r="J23" s="10">
         <f>IF(G23="","",SUM($G$8:G23))</f>
         <v/>
       </c>
@@ -1094,8 +1084,7 @@
       <c r="G24" s="10" t="n"/>
       <c r="H24" s="8" t="n"/>
       <c r="I24" s="8" t="n"/>
-      <c r="J24" s="8" t="n"/>
-      <c r="K24" s="10">
+      <c r="J24" s="10">
         <f>IF(G24="","",SUM($G$8:G24))</f>
         <v/>
       </c>
@@ -1116,8 +1105,7 @@
       <c r="G25" s="10" t="n"/>
       <c r="H25" s="8" t="n"/>
       <c r="I25" s="8" t="n"/>
-      <c r="J25" s="8" t="n"/>
-      <c r="K25" s="10">
+      <c r="J25" s="10">
         <f>IF(G25="","",SUM($G$8:G25))</f>
         <v/>
       </c>
@@ -1138,8 +1126,7 @@
       <c r="G26" s="10" t="n"/>
       <c r="H26" s="8" t="n"/>
       <c r="I26" s="8" t="n"/>
-      <c r="J26" s="8" t="n"/>
-      <c r="K26" s="10">
+      <c r="J26" s="10">
         <f>IF(G26="","",SUM($G$8:G26))</f>
         <v/>
       </c>
@@ -1160,8 +1147,7 @@
       <c r="G27" s="10" t="n"/>
       <c r="H27" s="8" t="n"/>
       <c r="I27" s="8" t="n"/>
-      <c r="J27" s="8" t="n"/>
-      <c r="K27" s="10">
+      <c r="J27" s="10">
         <f>IF(G27="","",SUM($G$8:G27))</f>
         <v/>
       </c>
@@ -1182,8 +1168,7 @@
       <c r="G28" s="10" t="n"/>
       <c r="H28" s="8" t="n"/>
       <c r="I28" s="8" t="n"/>
-      <c r="J28" s="8" t="n"/>
-      <c r="K28" s="10">
+      <c r="J28" s="10">
         <f>IF(G28="","",SUM($G$8:G28))</f>
         <v/>
       </c>
@@ -1204,8 +1189,7 @@
       <c r="G29" s="10" t="n"/>
       <c r="H29" s="8" t="n"/>
       <c r="I29" s="8" t="n"/>
-      <c r="J29" s="8" t="n"/>
-      <c r="K29" s="10">
+      <c r="J29" s="10">
         <f>IF(G29="","",SUM($G$8:G29))</f>
         <v/>
       </c>
@@ -1226,8 +1210,7 @@
       <c r="G30" s="10" t="n"/>
       <c r="H30" s="8" t="n"/>
       <c r="I30" s="8" t="n"/>
-      <c r="J30" s="8" t="n"/>
-      <c r="K30" s="10">
+      <c r="J30" s="10">
         <f>IF(G30="","",SUM($G$8:G30))</f>
         <v/>
       </c>
@@ -1248,8 +1231,7 @@
       <c r="G31" s="10" t="n"/>
       <c r="H31" s="8" t="n"/>
       <c r="I31" s="8" t="n"/>
-      <c r="J31" s="8" t="n"/>
-      <c r="K31" s="10">
+      <c r="J31" s="10">
         <f>IF(G31="","",SUM($G$8:G31))</f>
         <v/>
       </c>
@@ -1270,8 +1252,7 @@
       <c r="G32" s="10" t="n"/>
       <c r="H32" s="8" t="n"/>
       <c r="I32" s="8" t="n"/>
-      <c r="J32" s="8" t="n"/>
-      <c r="K32" s="10">
+      <c r="J32" s="10">
         <f>IF(G32="","",SUM($G$8:G32))</f>
         <v/>
       </c>
@@ -1292,8 +1273,7 @@
       <c r="G33" s="10" t="n"/>
       <c r="H33" s="8" t="n"/>
       <c r="I33" s="8" t="n"/>
-      <c r="J33" s="8" t="n"/>
-      <c r="K33" s="10">
+      <c r="J33" s="10">
         <f>IF(G33="","",SUM($G$8:G33))</f>
         <v/>
       </c>
@@ -1314,8 +1294,7 @@
       <c r="G34" s="10" t="n"/>
       <c r="H34" s="8" t="n"/>
       <c r="I34" s="8" t="n"/>
-      <c r="J34" s="8" t="n"/>
-      <c r="K34" s="10">
+      <c r="J34" s="10">
         <f>IF(G34="","",SUM($G$8:G34))</f>
         <v/>
       </c>
@@ -1336,8 +1315,7 @@
       <c r="G35" s="10" t="n"/>
       <c r="H35" s="8" t="n"/>
       <c r="I35" s="8" t="n"/>
-      <c r="J35" s="8" t="n"/>
-      <c r="K35" s="10">
+      <c r="J35" s="10">
         <f>IF(G35="","",SUM($G$8:G35))</f>
         <v/>
       </c>
@@ -1348,11 +1326,11 @@
           <t>TOTAL REFERRAL FEES PAID (RM)</t>
         </is>
       </c>
-      <c r="B36" s="8" t="n"/>
-      <c r="C36" s="8" t="n"/>
-      <c r="D36" s="8" t="n"/>
-      <c r="E36" s="8" t="n"/>
-      <c r="F36" s="8" t="n"/>
+      <c r="B36" s="17" t="n"/>
+      <c r="C36" s="17" t="n"/>
+      <c r="D36" s="17" t="n"/>
+      <c r="E36" s="17" t="n"/>
+      <c r="F36" s="18" t="n"/>
       <c r="G36" s="12">
         <f>SUM(G8:G35)</f>
         <v/>
@@ -1360,12 +1338,12 @@
       <c r="H36" s="8" t="n"/>
       <c r="I36" s="8" t="n"/>
       <c r="J36" s="8" t="n"/>
-      <c r="K36" s="8" t="n"/>
-    </row>
+    </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>Yellow rows are SAMPLES — delete and replace with your actual entries. No., Voucher No. and Running Total fill in automatically when you enter a Payee and Amount.</t>
+          <t>Yellow rows are SAMPLES, delete and replace with your actual entries. No., Voucher No. and Running Total fill in automatically when you enter a Payee and Amount.</t>
         </is>
       </c>
     </row>
@@ -1378,11 +1356,6 @@
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="H8:H35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Cash,Cheque,Bank Transfer"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1424,6 +1397,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -1431,17 +1405,19 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Voucher No.:</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>PV/2026/001</t>
         </is>
       </c>
+      <c r="C7" s="22" t="n"/>
       <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Date:</t>
@@ -1453,38 +1429,46 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Paid To:</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>Caryn</t>
         </is>
       </c>
-    </row>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
+    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
           <t>IC / Passport / Reg No.:</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="23" t="inlineStr">
         <is>
           <t>xxxxxx-xx-xxxx</t>
         </is>
       </c>
-    </row>
+      <c r="D11" s="22" t="n"/>
+      <c r="E11" s="22" t="n"/>
+    </row>
+    <row r="12"/>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>Address:</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr"/>
-    </row>
+      <c r="A13" s="14" t="n"/>
+      <c r="B13" s="23" t="inlineStr"/>
+      <c r="C13" s="22" t="n"/>
+      <c r="D13" s="22" t="n"/>
+      <c r="E13" s="22" t="n"/>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
@@ -1512,14 +1496,14 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Referral fee for Umesh Phadke — AB-39-02 MK 10</t>
+          <t>Referral fee for Umesh Phadke, AB-39-02 MK 10</t>
         </is>
       </c>
       <c r="C16" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="18" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="19" t="inlineStr">
@@ -1529,8 +1513,8 @@
       </c>
       <c r="B17" s="8" t="inlineStr"/>
       <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="n"/>
+      <c r="D17" s="17" t="n"/>
+      <c r="E17" s="18" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="19" t="inlineStr">
@@ -1540,8 +1524,8 @@
       </c>
       <c r="B18" s="8" t="inlineStr"/>
       <c r="C18" s="8" t="n"/>
-      <c r="D18" s="8" t="n"/>
-      <c r="E18" s="8" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="18" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -1549,50 +1533,39 @@
           <t>TOTAL (RM)</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n"/>
+      <c r="B19" s="18" t="n"/>
       <c r="C19" s="12">
         <f>SUM(C16:C18)</f>
         <v/>
       </c>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="n"/>
-    </row>
+      <c r="D19" s="17" t="n"/>
+      <c r="E19" s="18" t="n"/>
+    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Ringgit Malaysia (in words):</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="23" t="inlineStr">
         <is>
           <t>Two Thousand Only</t>
         </is>
       </c>
-    </row>
+      <c r="C21" s="22" t="n"/>
+      <c r="D21" s="22" t="n"/>
+      <c r="E21" s="22" t="n"/>
+    </row>
+    <row r="22"/>
     <row r="23">
-      <c r="A23" s="14" t="inlineStr">
-        <is>
-          <t>Payment Method:</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Bank Transfer</t>
-        </is>
-      </c>
+      <c r="A23" s="14" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>Cheque / Ref No.:</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>TXN12345</t>
-        </is>
-      </c>
-    </row>
+      <c r="A24" s="14" t="n"/>
+    </row>
+    <row r="25"/>
+    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
@@ -1627,6 +1600,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
@@ -1694,6 +1668,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -1701,17 +1676,19 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Receipt No.:</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>OR/2026/001</t>
         </is>
       </c>
+      <c r="C7" s="22" t="n"/>
       <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Date:</t>
@@ -1723,18 +1700,23 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Received From:</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>Kommons Realty Sdn Bhd</t>
         </is>
       </c>
-    </row>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
+    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
@@ -1743,12 +1725,17 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>Two Thousand Only</t>
         </is>
       </c>
-    </row>
+      <c r="B12" s="22" t="n"/>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="22" t="n"/>
+      <c r="E12" s="22" t="n"/>
+    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
@@ -1758,31 +1745,31 @@
       <c r="B14" s="12" t="n">
         <v>2000</v>
       </c>
-    </row>
+      <c r="C14" s="18" t="n"/>
+    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Being Payment For:</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>Referral fee — Umesh Phadke (AB-39-02 MK 10)</t>
-        </is>
-      </c>
-    </row>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>Referral fee, Umesh Phadke (AB-39-02 MK 10)</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="n"/>
+      <c r="D16" s="22" t="n"/>
+      <c r="E16" s="22" t="n"/>
+    </row>
+    <row r="17"/>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>Payment Method:</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Bank Transfer — Ref TXN12345</t>
-        </is>
-      </c>
-    </row>
+      <c r="A18" s="14" t="n"/>
+    </row>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22">
       <c r="D22" t="inlineStr">
         <is>
@@ -1804,10 +1791,12 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
+    <row r="26"/>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="21" t="inlineStr">
         <is>
-          <t>For LHDN: keep the referrer’s IC/Reg No. Referral fees to non-residents may attract withholding tax — confirm with your tax agent.</t>
+          <t>For LHDN: keep the referrer’s IC/Reg No. Referral fees to non-residents may attract withholding tax, confirm with your tax agent.</t>
         </is>
       </c>
     </row>

</xml_diff>